<commit_message>
fix(supply): correct KGEN circulating classification
</commit_message>
<xml_diff>
--- a/KGEN/registry/CoinMarketCap/KGEN_CMC_ANNEX_A_RICH_LIST_AND_RESERVES_V1.xlsx
+++ b/KGEN/registry/CoinMarketCap/KGEN_CMC_ANNEX_A_RICH_LIST_AND_RESERVES_V1.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annex A" sheetId="1" r:id="R7350a939480a4903"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation" sheetId="2" r:id="R2b5577fa0cc44a29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R1da3f9244c8d4744"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annex A" sheetId="1" r:id="R26e2a4a34a894f2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation" sheetId="2" r:id="R928e96b7cfa9482a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Rc58e55c14a6e4685"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -886,19 +886,19 @@
         <x:v>1.0216355936342444%</x:v>
       </x:c>
       <x:c r="E8" s="27" t="str">
-        <x:v>Unclassified major holder</x:v>
+        <x:v>Ownership-unverified major holder</x:v>
       </x:c>
       <x:c r="F8" s="27" t="str">
-        <x:v>UNKNOWN</x:v>
+        <x:v>PUBLIC_CIRCULATING</x:v>
       </x:c>
       <x:c r="G8" s="27" t="str">
-        <x:v>NON_CIRCULATING</x:v>
+        <x:v>CIRCULATING</x:v>
       </x:c>
       <x:c r="H8" s="27" t="str">
-        <x:v>EXCLUDED</x:v>
+        <x:v>INCLUDED</x:v>
       </x:c>
       <x:c r="I8" s="27" t="str">
-        <x:v>Public-float and control evidence not recorded</x:v>
+        <x:v>No evidence of project control, lock, vesting or non-circulation</x:v>
       </x:c>
       <x:c r="J8" s="27" t="str">
         <x:v>NOT_EVIDENCED</x:v>
@@ -907,13 +907,13 @@
         <x:v>NOT_EVIDENCED</x:v>
       </x:c>
       <x:c r="L8" s="27" t="str">
-        <x:v>UNKNOWN</x:v>
+        <x:v>OWNERSHIP_UNVERIFIED</x:v>
       </x:c>
       <x:c r="M8" s="27" t="str">
         <x:v>https://bscscan.com/token/0xba3d3810e58735cb6813bc1cdc5458c0d71432be?a=0xb73d6716005b37bec742d64482fa26033ee1a4e1</x:v>
       </x:c>
       <x:c r="N8" s="27" t="str">
-        <x:v>Excluded conservatively</x:v>
+        <x:v>Included under evidence-based classification</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" hidden="0" customHeight="1">
@@ -933,19 +933,19 @@
         <x:v>1.0210947223572304%</x:v>
       </x:c>
       <x:c r="E9" s="27" t="str">
-        <x:v>Unclassified major holder</x:v>
+        <x:v>Ownership-unverified major holder</x:v>
       </x:c>
       <x:c r="F9" s="27" t="str">
-        <x:v>UNKNOWN</x:v>
+        <x:v>PUBLIC_CIRCULATING</x:v>
       </x:c>
       <x:c r="G9" s="27" t="str">
-        <x:v>NON_CIRCULATING</x:v>
+        <x:v>CIRCULATING</x:v>
       </x:c>
       <x:c r="H9" s="27" t="str">
-        <x:v>EXCLUDED</x:v>
+        <x:v>INCLUDED</x:v>
       </x:c>
       <x:c r="I9" s="27" t="str">
-        <x:v>Public-float and control evidence not recorded</x:v>
+        <x:v>No evidence of project control, lock, vesting or non-circulation</x:v>
       </x:c>
       <x:c r="J9" s="27" t="str">
         <x:v>NOT_EVIDENCED</x:v>
@@ -954,13 +954,13 @@
         <x:v>NOT_EVIDENCED</x:v>
       </x:c>
       <x:c r="L9" s="27" t="str">
-        <x:v>UNKNOWN</x:v>
+        <x:v>OWNERSHIP_UNVERIFIED</x:v>
       </x:c>
       <x:c r="M9" s="27" t="str">
         <x:v>https://bscscan.com/token/0xba3d3810e58735cb6813bc1cdc5458c0d71432be?a=0xef83804c264b47378fcf150086943b53fb90a90b</x:v>
       </x:c>
       <x:c r="N9" s="27" t="str">
-        <x:v>Excluded conservatively</x:v>
+        <x:v>Included under evidence-based classification</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="24" hidden="0" customHeight="1">
@@ -1007,7 +1007,7 @@
         <x:v>https://bscscan.com/token/0xba3d3810e58735cb6813bc1cdc5458c0d71432be#balances</x:v>
       </x:c>
       <x:c r="N10" s="27" t="str">
-        <x:v>Aggregate derived as circulating supply minus public AMM liquidity</x:v>
+        <x:v>Aggregate excludes separately listed public AMM and ownership-unverified major holders</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="24" hidden="0" customHeight="1">
@@ -1171,7 +1171,7 @@
         <x:v>Circulating supply</x:v>
       </x:c>
       <x:c r="B7" s="51" t="str">
-        <x:v>2896511.372639273602111511</x:v>
+        <x:v>4366878.985936300061217422</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -1179,7 +1179,7 @@
         <x:v>Excluded balances</x:v>
       </x:c>
       <x:c r="B8" s="51" t="str">
-        <x:v>69083994.413478552101529489</x:v>
+        <x:v>67613626.800181525642423578</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -1243,13 +1243,13 @@
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="61" t="str">
-        <x:v>Unknown major holders</x:v>
+        <x:v>Ownership-unverified major holders</x:v>
       </x:c>
       <x:c r="B15" s="61" t="str">
-        <x:v>Excluded conservatively</x:v>
+        <x:v>Included in circulation</x:v>
       </x:c>
       <x:c r="C15" s="61" t="str">
-        <x:v>PR #55 methodology</x:v>
+        <x:v>Evidence-based classification</x:v>
       </x:c>
       <x:c r="D15" s="64" t="str">
         <x:v>VERIFIED</x:v>

</xml_diff>